<commit_message>
update import templates for departments and employees
</commit_message>
<xml_diff>
--- a/public/assets/import-templates/import-departments-template.xlsx
+++ b/public/assets/import-templates/import-departments-template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Source\Repos\mujd\frontend\public\assets\import-templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\3pillars\Repos\mujdn-frontend\public\assets\import-templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD135E15-5EBB-4587-92A0-35BED4863973}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA4F3832-6E99-4AA3-951F-772BFEC0B023}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C53C46E6-3CBA-4E34-9CE4-2BA44FFD488E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C53C46E6-3CBA-4E34-9CE4-2BA44FFD488E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -61,7 +61,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -71,6 +71,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -87,11 +93,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -407,19 +414,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CAE079F-3D3E-482A-8316-F8681F6A4CBD}">
   <dimension ref="A1:G1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.6328125" customWidth="1"/>
-    <col min="2" max="2" width="16.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.5703125" customWidth="1"/>
+    <col min="2" max="2" width="16.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="20" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.81640625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="21.81640625" customWidth="1"/>
+    <col min="6" max="6" width="19.85546875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="21.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">

</xml_diff>